<commit_message>
Keep Corp Pool Excel ingest working in production and stop Active List files landing in Resumes.
Deleted employees stay tombstoned, portal workbooks live in excel/, and 50656BR/50657BR cannot come back.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/BR/BR_RawData 3.xlsx
+++ b/docs/BR/BR_RawData 3.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="53">
   <si>
     <t>Auto req ID</t>
   </si>
@@ -86,6 +86,652 @@
   </si>
   <si>
     <t>ST (Bill Rate) Enter only numeric value and 0 for Non-Billable</t>
+  </si>
+  <si>
+    <t>50655BR</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>E2</t>
+  </si>
+  <si>
+    <t>Senior Software Engineer</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Technical</t>
+  </si>
+  <si>
+    <t>ITS - TMH - Delivery</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>SQL, Windows, Kafka, Java, Springboot, Hibernate, Spring Boot, Azure, Git</t>
+  </si>
+  <si>
+    <t>OFFSHORE</t>
+  </si>
+  <si>
+    <t>IRON MOUNTAIN</t>
+  </si>
+  <si>
+    <t>Billable</t>
+  </si>
+  <si>
+    <t>IM DXP-IDP 2025</t>
+  </si>
+  <si>
+    <t>1026374</t>
+  </si>
+  <si>
+    <t>Antony, Nithin (1027544)</t>
+  </si>
+  <si>
+    <t>Hippargi, Anil (1017237)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID: 50655BR 
+Status: Approved 
+Template: Infinite Standard Requisition 
+Languages 
+English (US) 
+Actions 
+Open Delete 
+eLink 
+View Approvals 
+Print 
+50655BR - Senior Software Engineer
+Status: Approved Job req template: Infinite Standard Requisition 
+One or more fields require your attention 
+Edit 
+Hold 
+Cancel 
+More 
+Details 
+History 
+Forms 
+Notes 
+*Job Code : 
+123456 Generic Job code
+Basic Information 
+*Entity : 
+Infinite Computer Solutions (India) Limited
+*SBU : 
+CMdS
+*Grade : 
+E3
+*Client Required Date : 
+12-Aug-2026
+*TAG / RMG Manager : 
+Singh, Ramendra (1025407)
+*Requirement Type : 
+New
+Comments : 
+*Backfill for Employee Name : 
+*Backfill Employee ID : 
+*Bill Rate Currency : 
+USD
+*Client Name : 
+Conduent Business Services LLC
+*BU : 
+Enterprise Technology Solutions
+*Sourcing Type : 
+Internal
+Date Moved : 
+*Designation : 
+Senior Software Engineer
+*Designation (US) : 
+*Title : 
+Senior Software Engineer
+*Employment type : 
+Employee
+Job Type : 
+*EmployeeSubType : 
+Lateral/ New Hire
+*Employment Class : 
+*Job description : 
+Java Senior Developer (C06) – Job DescriptionA software developer who
+Engage in application development, test, release and support.
+Produce fully functional application code based on industry best practices.
+Gather specific requirements, ask questions and suggest solutions.
+Write unit and API tests to ensure working code and support CICD team.
+Troubleshoot and debug to optimize performance.
+Liaise with the Product development team to plan new features in agile model.
+Ensure applications meet quality standards.
+Basic Qualifications:
+Bachelor’s degree in Computer Science, Information Technology, or a similar field.
+3-6 years of overall IT experience
+Hands-on Experience as a Java Developer 
+2+ years’ experience with Spring/Springboot &amp; ORM 
+2 years’ experience with middleware / service orchestration
+Experience with performance optimization, performance testing/monitoring tools experience 
+Experience with common industry patterns, coding standards and best practices
+Excellent troubleshooting skills.
+Excellent written &amp; verbal communication.
+Technical Skills &amp; Qualifications:
+Required - Java, Spring, Spring Boot, Spring MVC, Hibernate/Spring JPA, SQL, GIT
+Good to have - Apache Kafka/RabbitMQ, MongoDb, Azure DevOps, Git
+Preferred Qualifications for Consideration:
+Healthcare experience preferred
+Experience with mentoring and training junior associates
+Experience working in large development team
+*Project : 
+Conduent - CMdS Product Automation Testing
+*Business Group : 
+Delivery
+*Department Type : 
+Technical
+*No. of Positions : 
+1
+*Position Reporting to : 
+Samantara, Radhakanta (1010164)
+*Manager Employee ID : 
+1010164
+*Requester ID : 
+1010164
+*Req team : 
+Louis, Diana (1006001)
+Ramamurthy, Srinath (1022501)
+Singh, Ramendra (1025407)
+Patel, Alpa (1024167)
+Shruthi, S (1027249)
+Andrews, Alden (1028556)
+Baggam, Asha (1026370)
+Bharath, Shwetha (1037293)
+Jha, Rashmi (1037981)
+Jayakumar, Monish (1039455)
+Reddy, Nehalatha (1043618)
+*Billing Type : 
+Billable
+*Bill Rate Type : 
+Hourly
+Target Rate (Agency) : 
+*ST (Bill Rate) Enter only numeric value and 0 for Non-Billable : 
+24
+*OT : 
+Project Duration (In months) : 
+*Contract Duration : 
+*End Date : 
+Costa Rica Specific Fields 
+Job Group : 
+Progression : 
+Position ID : 
+Job Family : 
+Management Level : 
+Track : 
+Position Budget (in $) : 
+Detail Information 
+*Notice Period (In Days) : 
+60
+*Physical Location : 
+Bangalore
+Job City : 
+*Qualifications / Degree : 
+BE
+Target Companies : 
+Other Comments : 
+Bangalore/Hyderabad
+*Range of Year Experience-Min Year : 
+4
+*Mandatory Skills1 : 
+Java
+Java Spring boot
+Hibernate
+*Mandatory Skills2 : 
+*Mandatory Skills3 : 
+*Branch / Major : 
+CS
+*Unit Location : 
+Bangalore - Campus
+*Range of Year Experience-Max Year : 
+8
+*Handling a Team : 
+Eventually
+Trainable Skill : 
+*Joining Location : 
+Hyderabad
+Interview Details 
+*MSA Contract Signed : 
+Yes
+*Expected Sign Date : 
+SOW signed : 
+N/A
+*Client Interview? : 
+Yes
+Client Interview Details : 
+*Type of Pooling : 
+External
+Comments/Reason : 
+*Background Check : 
+Post
+IT &amp; Admin Service Requirements 
+*Work Station : 
+Required
+*Required Laptop Configuration : 
+Standard Infinite Laptop with Infinite Image(I5 / 16 GB / 512 GB SSD / Windows 11 Pro)
+*Non-Standard Laptop Configuration : 
+*MS Office Request : 
+Not Required
+*VOIP : 
+Not Required
+VOIP Addititonal Info : 
+*VOIP Plan Duration 1501 : 
+*VOIP Plan Duration 2622 : 
+Request has to be raised in Service Management Module
+Turn off Autofiler notification for this req 
+For internal use only 
+Client Name/Code : 
+Conduent Business Services LLC/253
+Project/Code : 
+Conduent - CMdS Product Au</t>
+  </si>
+  <si>
+    <t>Bangalore - Global Axis</t>
+  </si>
+  <si>
+    <t>2026-08-25</t>
+  </si>
+  <si>
+    <t>External - India</t>
+  </si>
+  <si>
+    <t>New</t>
+  </si>
+  <si>
+    <t>50944BR</t>
+  </si>
+  <si>
+    <t>Technical Lead</t>
+  </si>
+  <si>
+    <t>SQL, Windows, Python, React, AWS, Azure, Jira, ServiceNow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID: 50944BR 
+Status: Approved 
+Template: Infinite Standard Requisition 
+Languages 
+English (US) 
+Actions 
+Open Delete 
+eLink 
+View Approvals 
+Print 
+50944BR - Technical Lead
+Status: Approved Job req template: Infinite Standard Requisition 
+One or more fields require your attention 
+Edit 
+Hold 
+Cancel 
+More 
+Details 
+History 
+Forms 
+Notes 
+*Job Code : 
+123456 Generic Job code
+Basic Information 
+*Entity : 
+Infinite Computer Solutions (India) Limited
+*SBU : 
+FiServ
+*Grade : 
+E4
+*Client Required Date : 
+19-Aug-2026
+*TAG / RMG Manager : 
+Singh, Ramendra (1025407)
+*Requirement Type : 
+New
+Comments : 
+*Backfill for Employee Name : 
+*Backfill Employee ID : 
+*Bill Rate Currency : 
+USD
+*Client Name : 
+Fiserv Solutions, LLC
+*BU : 
+Enterprise Technology Solutions
+*Sourcing Type : 
+Internal
+Date Moved : 
+*Designation : 
+Technical Lead
+*Designation (US) : 
+*Title : 
+Technical Lead
+*Employment type : 
+Employee
+Job Type : 
+*EmployeeSubType : 
+Lateral/ New Hire
+*Employment Class : 
+*Job description : 
+Requirements: 
+5+ years of experience in software development, with a strong focus on .NET technologies, including Web API.
+Solid understanding of SQL and database design and management. 
+Familiarity with REST API fundamentals. 
+Excellent problem-solving skills and the ability to work in a fast-paced environment. 
+Strong communication skills to effectively collaborate with cross-functional teams. 
+Good understanding of software development principles and design patterns. 
+Exposure to cloud platforms like Azure or AWS.
+Nice to Have: 
+Extensive experience with Azure cloud. 
+Familiarity with machine learning concepts and Python programming.
+Familiarity with UI development using React  
+Knowledge of DevOps practices and CI/CD pipelines.
+*Project : 
+Fiserv - Data Services Support
+*Business Group : 
+Delivery
+*Department Type : 
+Technical
+*No. of Positions : 
+1
+*Position Reporting to : 
+Prasad, Kali (1040272)
+*Manager Employee ID : 
+1040272
+*Requester ID : 
+1040272
+*Req team : 
+Louis, Diana (1006001)
+Ramamurthy, Srinath (1022501)
+Singh, Ramendra (1025407)
+Patel, Alpa (1024167)
+Shruthi, S (1027249)
+Andrews, Alden (1028556)
+Baggam, Asha (1026370)
+Bharath, Shwetha (1037293)
+Jha, Rashmi (1037981)
+Jayakumar, Monish (1039455)
+Reddy, Nehalatha (1043618)
+*Billing Type : 
+Billable
+*Bill Rate Type : 
+Hourly
+Target Rate (Agency) : 
+*ST (Bill Rate) Enter only numeric value and 0 for Non-Billable : 
+41.71
+*OT : 
+Project Duration (In months) : 
+*Contract Duration : 
+*End Date : 
+Costa Rica Specific Fields 
+Job Group : 
+Progression : 
+Position ID : 
+Job Family : 
+Management Level : 
+Track : 
+Position Budget (in $) : 
+Detail Information 
+*Notice Period (In Days) : 
+60
+*Physical Location : 
+Pune
+Job City : 
+*Qualifications / Degree : 
+BE
+Target Companies : 
+Other Comments : 
+*Range of Year Experience-Min Year : 
+5
+*Mandatory Skills1 : 
+.NET
+*Mandatory Skills2 : 
+Azure Data Bricks
+*Mandatory Skills3 : 
+Web API
+*Branch / Major : 
+CS
+*Unit Location : 
+Bangalore - Campus
+*Range of Year Experience-Max Year : 
+8
+*Handling a Team : 
+Eventually
+Trainable Skill : 
+*Joining Location : 
+Pune
+Interview Details 
+*MSA Contract Signed : 
+Yes
+*Expected Sign Date : 
+SOW signed : 
+N/A
+*Client Interview? : 
+Yes
+Client Interview Details : 
+*Type of Pooling : 
+External
+Comments/Reason : 
+*Background Check : 
+Post
+IT &amp; Admin Service Requirements 
+*Work Station : 
+Required
+*Required Laptop Configuration : 
+Standard Infinite Laptop with Infinite Image(I5 / 16 GB / 512 GB SSD / Windows 11 Pro)
+*Non-Standard Laptop Configuration : 
+*MS Office Request : 
+Not Required
+*VOIP : 
+Not Required
+VOIP Addititonal Info : 
+*VOIP Plan Duration 1501 : 
+*VOIP Plan Duration 2622 : 
+Request has to be raised in Service Management Module
+Turn off Autofiler notification for this req 
+For internal use only 
+Client Name/Code : 
+Fiserv Solutions, LLC/1360
+Project/Code : 
+17103188/Fiserv - Data Services Support
+SBU/Code : 
+FiServ/42271
+BU/Code : 
+Enterprise Technology Solutions/42251
+Job State : 
+Job Country : 
+IN
+Req ID : 
+Print
+</t>
+  </si>
+  <si>
+    <t>50744BR</t>
+  </si>
+  <si>
+    <t>Windows, Jira, ServiceNow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID: 50744BR 
+Status: Approved 
+Template: Infinite Standard Requisition 
+Languages 
+English (US) 
+Actions 
+Open Delete 
+eLink 
+View Approvals 
+Print 
+50744BR - Senior Software Engineer
+Status: Approved Job req template: Infinite Standard Requisition 
+One or more fields require your attention 
+Edit 
+Hold 
+Cancel 
+More 
+Details 
+History 
+Forms 
+Notes 
+*Job Code : 
+123456 Generic Job code
+Basic Information 
+*Entity : 
+Infinite Computer Solutions (India) Limited
+*SBU : 
+FiServ
+*Grade : 
+E3
+*Client Required Date : 
+13-Aug-2026
+*TAG / RMG Manager : 
+Singh, Ramendra (1025407)
+*Requirement Type : 
+Backfill
+Comments : 
+*Backfill for Employee Name : 
+Roshan Lomga
+*Backfill Employee ID : 
+1032459
+*Bill Rate Currency : 
+USD
+*Client Name : 
+Fiserv Solutions, LLC
+*BU : 
+Enterprise Technology Solutions
+*Sourcing Type : 
+Internal
+Date Moved : 
+*Designation : 
+Senior Software Engineer
+*Designation (US) : 
+*Title : 
+Senior Software Engineer
+*Employment type : 
+Employee
+Job Type : 
+*EmployeeSubType : 
+Lateral/ New Hire
+*Employment Class : 
+*Job description : 
+Senior Software Engineer with 4+ years of experience
+*Project : 
+Fiserv - Architect Professional Services
+*Business Group : 
+Delivery
+*Department Type : 
+Technical
+*No. of Positions : 
+1
+*Position Reporting to : 
+Kochunni, Nagarajan (1019672)
+*Manager Employee ID : 
+1019672
+*Requester ID : 
+1019672
+*Req team : 
+Louis, Diana (1006001)
+Ramamurthy, Srinath (1022501)
+Singh, Ramendra (1025407)
+Patel, Alpa (1024167)
+Shruthi, S (1027249)
+Andrews, Alden (1028556)
+Baggam, Asha (1026370)
+Bharath, Shwetha (1037293)
+Jha, Rashmi (1037981)
+Jayakumar, Monish (1039455)
+Reddy, Nehalatha (1043618)
+*Billing Type : 
+Billable
+*Bill Rate Type : 
+Hourly
+Target Rate (Agency) : 
+*ST (Bill Rate) Enter only numeric value and 0 for Non-Billable : 
+32.98
+*OT : 
+Project Duration (In months) : 
+*Contract Duration : 
+*End Date : 
+Costa Rica Specific Fields 
+Job Group : 
+Progression : 
+Position ID : 
+Job Family : 
+Management Level : 
+Track : 
+Position Budget (in $) : 
+Detail Information 
+*Notice Period (In Days) : 
+60
+*Physical Location : 
+Bangalore
+Job City : 
+*Qualifications / Degree : 
+BE
+Target Companies : 
+Other Comments : 
+*Range of Year Experience-Min Year : 
+4
+*Mandatory Skills1 : 
+.NET
+ASP.Net
+*Mandatory Skills2 : 
+*Mandatory Skills3 : 
+*Branch / Major : 
+CS
+*Unit Location : 
+Bangalore - Campus
+*Range of Year Experience-Max Year : 
+8
+*Handling a Team : 
+Eventually
+Trainable Skill : 
+*Joining Location : 
+Bangalore
+Interview Details 
+*MSA Contract Signed : 
+Yes
+*Expected Sign Date : 
+SOW signed : 
+N/A
+*Client Interview? : 
+Yes
+Client Interview Details : 
+*Type of Pooling : 
+External
+Comments/Reason : 
+*Background Check : 
+Post
+IT &amp; Admin Service Requirements 
+*Work Station : 
+Required
+*Required Laptop Configuration : 
+Standard Infinite Laptop with Infinite Image(I5 / 16 GB / 512 GB SSD / Windows 11 Pro)
+*Non-Standard Laptop Configuration : 
+*MS Office Request : 
+Not Required
+*VOIP : 
+Not Required
+VOIP Addititonal Info : 
+*VOIP Plan Duration 1501 : 
+*VOIP Plan Duration 2622 : 
+Request has to be raised in Service Management Module
+Turn off Autofiler notification for this req 
+For internal use only 
+Client Name/Code : 
+Fiserv Solutions, LLC/1360
+Project/Code : 
+Fiserv - Architect Professional Services/17101824
+SBU/Code : 
+FiServ/42271
+BU/Code : 
+Enterprise Technology Solutions/42251
+Job State : 
+Job Country : 
+IN
+Req ID : 
+Print
+</t>
   </si>
 </sst>
 </file>
@@ -462,7 +1108,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y1"/>
+  <dimension ref="A1:Y4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
@@ -542,8 +1188,230 @@
         <v>24</v>
       </c>
     </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L2" t="s">
+        <v>36</v>
+      </c>
+      <c r="M2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2" t="s">
+        <v>39</v>
+      </c>
+      <c r="P2" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>41</v>
+      </c>
+      <c r="R2" t="s">
+        <v>42</v>
+      </c>
+      <c r="T2" t="s">
+        <v>43</v>
+      </c>
+      <c r="U2">
+        <v>1</v>
+      </c>
+      <c r="V2">
+        <v>1</v>
+      </c>
+      <c r="W2" t="s">
+        <v>44</v>
+      </c>
+      <c r="X2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y2">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K3" t="s">
+        <v>35</v>
+      </c>
+      <c r="L3" t="s">
+        <v>36</v>
+      </c>
+      <c r="M3" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" t="s">
+        <v>38</v>
+      </c>
+      <c r="O3" t="s">
+        <v>39</v>
+      </c>
+      <c r="P3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>49</v>
+      </c>
+      <c r="R3" t="s">
+        <v>42</v>
+      </c>
+      <c r="T3" t="s">
+        <v>43</v>
+      </c>
+      <c r="U3">
+        <v>1</v>
+      </c>
+      <c r="V3">
+        <v>1</v>
+      </c>
+      <c r="W3" t="s">
+        <v>44</v>
+      </c>
+      <c r="X3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y3">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K4" t="s">
+        <v>35</v>
+      </c>
+      <c r="L4" t="s">
+        <v>36</v>
+      </c>
+      <c r="M4" t="s">
+        <v>37</v>
+      </c>
+      <c r="N4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4" t="s">
+        <v>39</v>
+      </c>
+      <c r="P4" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>52</v>
+      </c>
+      <c r="R4" t="s">
+        <v>42</v>
+      </c>
+      <c r="T4" t="s">
+        <v>43</v>
+      </c>
+      <c r="U4">
+        <v>1</v>
+      </c>
+      <c r="V4">
+        <v>1</v>
+      </c>
+      <c r="W4" t="s">
+        <v>44</v>
+      </c>
+      <c r="X4" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y4">
+        <v>5.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>